<commit_message>
Clean up Robot Arm repo structure and organize project files
</commit_message>
<xml_diff>
--- a/mechanical/bom/Robot_Arm_BOM.xlsx
+++ b/mechanical/bom/Robot_Arm_BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\Projects\Robot_Arm_\mechanical\bom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01613EE5-9367-48B7-8A4D-1A568596470E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11CF2420-614C-420C-B851-874E08190BEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-1020" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2295" yWindow="2295" windowWidth="28800" windowHeight="15885" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -70,9 +70,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>Some Amazon order totals include multiple items (e.g., $19.77 includes both inserts + M3 screw kit). If you want per-item exact costs, paste the invoice line-item prices and I can update.</t>
-  </si>
-  <si>
     <t>Robot Arm BOM – Purchased &amp; Owned</t>
   </si>
   <si>
@@ -632,6 +629,9 @@
   </si>
   <si>
     <t>Nema 23 Kit</t>
+  </si>
+  <si>
+    <t>Some Amazon order totals include multiple items (e.g., $19.77 includes both inserts + M3 screw kit). If you want per-item exact costs, paste the invoice line-item prices and I can update. This is a living BOM and will be subject to changes in the forseeable future.</t>
   </si>
 </sst>
 </file>
@@ -759,15 +759,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="8" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1149,7 +1149,7 @@
         <v>8</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>9</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -1177,58 +1177,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
+      <c r="A1" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
     </row>
     <row r="3" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="C3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="H3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="I3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="J3" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="K3" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="L3" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="L3" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="M3" s="6" t="s">
         <v>8</v>
@@ -1236,16 +1236,16 @@
     </row>
     <row r="4" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="C4" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>25</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>26</v>
       </c>
       <c r="E4" s="8">
         <v>1</v>
@@ -1256,37 +1256,37 @@
       <c r="G4" s="9">
         <v>9.49</v>
       </c>
-      <c r="H4" s="15">
+      <c r="H4" s="13">
         <v>9.49</v>
       </c>
       <c r="I4" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="J4" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="J4" s="7" t="s">
+      <c r="K4" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="K4" s="7" t="s">
+      <c r="L4" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="M4" s="7" t="s">
         <v>29</v>
-      </c>
-      <c r="L4" s="13" t="s">
-        <v>186</v>
-      </c>
-      <c r="M4" s="7" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="7" t="s">
-        <v>24</v>
-      </c>
       <c r="C5" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>31</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>32</v>
       </c>
       <c r="E5" s="8">
         <v>1</v>
@@ -1301,33 +1301,33 @@
         <v>8.99</v>
       </c>
       <c r="I5" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="J5" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="J5" s="7" t="s">
+      <c r="K5" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="L5" s="14" t="s">
-        <v>187</v>
+      <c r="L5" s="12" t="s">
+        <v>186</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="7" t="s">
-        <v>24</v>
-      </c>
       <c r="C6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>34</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>35</v>
       </c>
       <c r="E6" s="7">
         <v>1</v>
@@ -1342,33 +1342,33 @@
         <v>10.69</v>
       </c>
       <c r="I6" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="J6" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="J6" s="7" t="s">
-        <v>28</v>
-      </c>
       <c r="K6" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="L6" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="M6" s="7" t="s">
         <v>36</v>
-      </c>
-      <c r="L6" s="14" t="s">
-        <v>188</v>
-      </c>
-      <c r="M6" s="7" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="C7" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="D7" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="E7" s="8">
         <v>20</v>
@@ -1383,33 +1383,33 @@
         <v>6.99</v>
       </c>
       <c r="I7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="J7" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="J7" s="7" t="s">
-        <v>28</v>
-      </c>
       <c r="K7" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="L7" s="12" t="s">
+        <v>188</v>
+      </c>
+      <c r="M7" s="7" t="s">
         <v>42</v>
-      </c>
-      <c r="L7" s="14" t="s">
-        <v>189</v>
-      </c>
-      <c r="M7" s="7" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B8" s="7" t="s">
-        <v>39</v>
-      </c>
       <c r="C8" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>44</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>45</v>
       </c>
       <c r="E8" s="8">
         <v>2</v>
@@ -1424,33 +1424,33 @@
         <v>13.99</v>
       </c>
       <c r="I8" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="J8" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="J8" s="7" t="s">
-        <v>28</v>
-      </c>
       <c r="K8" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="L8" s="14" t="s">
-        <v>190</v>
+        <v>41</v>
+      </c>
+      <c r="L8" s="12" t="s">
+        <v>189</v>
       </c>
       <c r="M8" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B9" s="7" t="s">
-        <v>39</v>
-      </c>
       <c r="C9" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>47</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>48</v>
       </c>
       <c r="E9" s="8">
         <v>1</v>
@@ -1465,33 +1465,33 @@
         <v>9.49</v>
       </c>
       <c r="I9" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="J9" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="J9" s="7" t="s">
-        <v>28</v>
-      </c>
       <c r="K9" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="L9" s="14" t="s">
-        <v>191</v>
+        <v>41</v>
+      </c>
+      <c r="L9" s="12" t="s">
+        <v>190</v>
       </c>
       <c r="M9" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="7" t="s">
-        <v>39</v>
-      </c>
       <c r="C10" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>50</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>51</v>
       </c>
       <c r="E10" s="8">
         <v>6</v>
@@ -1506,33 +1506,33 @@
         <v>9.19</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>28</v>
+        <v>81</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="L10" s="14" t="s">
-        <v>192</v>
+        <v>41</v>
+      </c>
+      <c r="L10" s="12" t="s">
+        <v>191</v>
       </c>
       <c r="M10" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="C11" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="D11" s="7" t="s">
         <v>55</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>56</v>
       </c>
       <c r="E11" s="8">
         <v>5</v>
@@ -1547,33 +1547,33 @@
         <v>55</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J11" s="7" t="s">
-        <v>28</v>
+        <v>81</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="L11" s="14" t="s">
-        <v>193</v>
+        <v>41</v>
+      </c>
+      <c r="L11" s="12" t="s">
+        <v>192</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="C12" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="D12" s="7" t="s">
         <v>60</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>61</v>
       </c>
       <c r="E12" s="7">
         <v>5</v>
@@ -1588,33 +1588,33 @@
         <v>21.99</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>28</v>
+        <v>81</v>
       </c>
       <c r="K12" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="L12" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="M12" s="7" t="s">
         <v>62</v>
-      </c>
-      <c r="L12" s="14" t="s">
-        <v>194</v>
-      </c>
-      <c r="M12" s="7" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="C13" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="D13" s="7" t="s">
         <v>66</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>67</v>
       </c>
       <c r="E13" s="8">
         <v>1</v>
@@ -1629,33 +1629,33 @@
         <v>35.43</v>
       </c>
       <c r="I13" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="J13" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="K13" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="J13" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="K13" s="7" t="s">
+      <c r="L13" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="M13" s="7" t="s">
         <v>69</v>
-      </c>
-      <c r="L13" s="14" t="s">
-        <v>195</v>
-      </c>
-      <c r="M13" s="7" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="B14" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="C14" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="D14" s="7" t="s">
         <v>73</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>74</v>
       </c>
       <c r="E14" s="8">
         <v>1</v>
@@ -1670,71 +1670,71 @@
         <v>72.3</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>28</v>
+        <v>81</v>
       </c>
       <c r="K14" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="L14" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="M14" s="7" t="s">
         <v>75</v>
-      </c>
-      <c r="L14" s="14" t="s">
-        <v>196</v>
-      </c>
-      <c r="M14" s="7" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B15" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="C15" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="D15" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="E15" s="8">
+        <v>1</v>
+      </c>
+      <c r="F15" s="9">
+        <v>0</v>
+      </c>
+      <c r="G15" s="9">
+        <v>0</v>
+      </c>
+      <c r="H15" s="9">
+        <v>0</v>
+      </c>
+      <c r="I15" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="E15" s="8">
-        <v>1</v>
-      </c>
-      <c r="F15" s="9">
-        <v>0</v>
-      </c>
-      <c r="G15" s="9">
-        <v>0</v>
-      </c>
-      <c r="H15" s="9">
-        <v>0</v>
-      </c>
-      <c r="I15" s="7" t="s">
+      <c r="J15" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="J15" s="7" t="s">
+      <c r="K15" s="7"/>
+      <c r="L15" s="12"/>
+      <c r="M15" s="7" t="s">
         <v>82</v>
-      </c>
-      <c r="K15" s="7"/>
-      <c r="L15" s="14"/>
-      <c r="M15" s="7" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="B16" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="C16" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="D16" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="D16" s="7" t="s">
-        <v>87</v>
-      </c>
       <c r="E16" s="8">
         <v>1</v>
       </c>
@@ -1748,30 +1748,30 @@
         <v>0</v>
       </c>
       <c r="I16" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="J16" s="7" t="s">
         <v>81</v>
-      </c>
-      <c r="J16" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="K16" s="7"/>
       <c r="L16" s="7"/>
       <c r="M16" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="C17" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="D17" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="D17" s="7" t="s">
-        <v>92</v>
-      </c>
       <c r="E17" s="8">
         <v>1</v>
       </c>
@@ -1785,30 +1785,30 @@
         <v>0</v>
       </c>
       <c r="I17" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="J17" s="7" t="s">
         <v>81</v>
-      </c>
-      <c r="J17" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="K17" s="7"/>
       <c r="L17" s="7"/>
       <c r="M17" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B18" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="C18" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="D18" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="D18" s="7" t="s">
-        <v>97</v>
-      </c>
       <c r="E18" s="8">
         <v>1</v>
       </c>
@@ -1822,29 +1822,29 @@
         <v>0</v>
       </c>
       <c r="I18" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="J18" s="7" t="s">
         <v>81</v>
-      </c>
-      <c r="J18" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="K18" s="7"/>
       <c r="L18" s="7"/>
       <c r="M18" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="C19" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="D19" s="7" t="s">
         <v>101</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>102</v>
       </c>
       <c r="E19" s="8">
         <v>6</v>
@@ -1859,30 +1859,30 @@
         <v>0</v>
       </c>
       <c r="I19" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="J19" s="7" t="s">
         <v>81</v>
-      </c>
-      <c r="J19" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="K19" s="7"/>
       <c r="L19" s="7"/>
       <c r="M19" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B20" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="C20" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="D20" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="D20" s="7" t="s">
-        <v>107</v>
-      </c>
       <c r="E20" s="8">
         <v>1</v>
       </c>
@@ -1896,30 +1896,30 @@
         <v>0</v>
       </c>
       <c r="I20" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="J20" s="7" t="s">
         <v>81</v>
-      </c>
-      <c r="J20" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="K20" s="7"/>
       <c r="L20" s="7"/>
       <c r="M20" s="7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="B21" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="C21" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="D21" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="D21" s="7" t="s">
-        <v>112</v>
-      </c>
       <c r="E21" s="8">
         <v>1</v>
       </c>
@@ -1933,30 +1933,30 @@
         <v>0</v>
       </c>
       <c r="I21" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="J21" s="7" t="s">
         <v>81</v>
-      </c>
-      <c r="J21" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="K21" s="7"/>
       <c r="L21" s="7"/>
       <c r="M21" s="7" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="B22" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="C22" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="D22" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="D22" s="7" t="s">
-        <v>117</v>
-      </c>
       <c r="E22" s="7">
         <v>1</v>
       </c>
@@ -1970,30 +1970,30 @@
         <v>0</v>
       </c>
       <c r="I22" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="J22" s="7" t="s">
         <v>81</v>
-      </c>
-      <c r="J22" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="K22" s="7"/>
       <c r="L22" s="7"/>
       <c r="M22" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="C23" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="B23" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="C23" s="7" t="s">
+      <c r="D23" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="D23" s="7" t="s">
-        <v>121</v>
-      </c>
       <c r="E23" s="7">
         <v>1</v>
       </c>
@@ -2007,30 +2007,30 @@
         <v>0</v>
       </c>
       <c r="I23" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="J23" s="7" t="s">
         <v>81</v>
-      </c>
-      <c r="J23" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="K23" s="7"/>
       <c r="L23" s="7"/>
       <c r="M23" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C24" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="D24" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="D24" s="7" t="s">
-        <v>123</v>
-      </c>
       <c r="E24" s="7">
         <v>1</v>
       </c>
@@ -2044,30 +2044,30 @@
         <v>0</v>
       </c>
       <c r="I24" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="J24" s="7" t="s">
         <v>81</v>
-      </c>
-      <c r="J24" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="K24" s="7"/>
       <c r="L24" s="7"/>
       <c r="M24" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="C25" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="B25" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="C25" s="7" t="s">
+      <c r="D25" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="D25" s="7" t="s">
-        <v>126</v>
-      </c>
       <c r="E25" s="7">
         <v>1</v>
       </c>
@@ -2081,30 +2081,30 @@
         <v>0</v>
       </c>
       <c r="I25" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="J25" s="7" t="s">
         <v>81</v>
-      </c>
-      <c r="J25" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="K25" s="7"/>
       <c r="L25" s="7"/>
       <c r="M25" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="26" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C26" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="D26" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="D26" s="7" t="s">
-        <v>128</v>
-      </c>
       <c r="E26" s="7">
         <v>1</v>
       </c>
@@ -2118,30 +2118,30 @@
         <v>0</v>
       </c>
       <c r="I26" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="J26" s="7" t="s">
         <v>81</v>
-      </c>
-      <c r="J26" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="K26" s="7"/>
       <c r="L26" s="7"/>
       <c r="M26" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="C27" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="B27" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="C27" s="7" t="s">
+      <c r="D27" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="D27" s="7" t="s">
-        <v>131</v>
-      </c>
       <c r="E27" s="7">
         <v>1</v>
       </c>
@@ -2155,15 +2155,15 @@
         <v>0</v>
       </c>
       <c r="I27" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="J27" s="7" t="s">
         <v>81</v>
-      </c>
-      <c r="J27" s="7" t="s">
-        <v>82</v>
       </c>
       <c r="K27" s="7"/>
       <c r="L27" s="7"/>
       <c r="M27" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
@@ -2171,7 +2171,7 @@
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
       <c r="D28" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E28" s="7"/>
       <c r="F28" s="7"/>
@@ -2225,46 +2225,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
-        <v>133</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
+      <c r="A1" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="C3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="6" t="s">
-        <v>15</v>
-      </c>
       <c r="F3" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="H3" s="6" t="s">
-        <v>20</v>
-      </c>
       <c r="I3" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J3" s="6" t="s">
         <v>8</v>
@@ -2272,47 +2272,47 @@
     </row>
     <row r="4" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="C4" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="E4" s="7">
+        <v>1</v>
+      </c>
+      <c r="F4" s="9">
+        <v>0</v>
+      </c>
+      <c r="G4" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="E4" s="7">
-        <v>1</v>
-      </c>
-      <c r="F4" s="9">
-        <v>0</v>
-      </c>
-      <c r="G4" s="7" t="s">
+      <c r="H4" s="7" t="s">
         <v>139</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>140</v>
       </c>
       <c r="I4" s="7"/>
       <c r="J4" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B5" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="C5" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="D5" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="D5" s="7" t="s">
-        <v>144</v>
-      </c>
       <c r="E5" s="7">
         <v>1</v>
       </c>
@@ -2320,29 +2320,29 @@
         <v>0</v>
       </c>
       <c r="G5" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="H5" s="7" t="s">
         <v>139</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>140</v>
       </c>
       <c r="I5" s="7"/>
       <c r="J5" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B6" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="D6" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>148</v>
-      </c>
       <c r="E6" s="7">
         <v>1</v>
       </c>
@@ -2350,14 +2350,14 @@
         <v>0</v>
       </c>
       <c r="G6" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="H6" s="7" t="s">
         <v>139</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>140</v>
       </c>
       <c r="I6" s="7"/>
       <c r="J6" s="7" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -2365,7 +2365,7 @@
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
       <c r="D7" s="7" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E7" s="7"/>
       <c r="F7" s="9">
@@ -2400,42 +2400,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
+      <c r="A1" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="C3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="6" t="s">
-        <v>15</v>
-      </c>
       <c r="F3" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I3" s="6" t="s">
         <v>8</v>
@@ -2443,16 +2443,16 @@
     </row>
     <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="B4" s="7" t="s">
-        <v>90</v>
-      </c>
       <c r="C4" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>153</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>154</v>
       </c>
       <c r="E4" s="8">
         <v>1</v>
@@ -2461,27 +2461,27 @@
         <v>12</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H4" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="I4" s="7" t="s">
         <v>155</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C5" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>157</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>158</v>
       </c>
       <c r="E5" s="8">
         <v>1</v>
@@ -2490,27 +2490,27 @@
         <v>6</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B6" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="D6" s="7" t="s">
         <v>161</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>162</v>
       </c>
       <c r="E6" s="8">
         <v>1</v>
@@ -2519,27 +2519,27 @@
         <v>25</v>
       </c>
       <c r="G6" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="I6" s="7" t="s">
         <v>163</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B7" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="C7" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="D7" s="7" t="s">
         <v>166</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>167</v>
       </c>
       <c r="E7" s="8">
         <v>1</v>
@@ -2548,25 +2548,25 @@
         <v>15</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I7" s="7"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="C8" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="D8" s="7" t="s">
         <v>170</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>171</v>
       </c>
       <c r="E8" s="8">
         <v>6</v>
@@ -2575,27 +2575,27 @@
         <v>10</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="B9" s="7" t="s">
-        <v>105</v>
-      </c>
       <c r="C9" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>173</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>174</v>
       </c>
       <c r="E9" s="8">
         <v>1</v>
@@ -2604,25 +2604,25 @@
         <v>20</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I9" s="7"/>
     </row>
     <row r="10" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B10" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="C10" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="D10" s="7" t="s">
         <v>176</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>177</v>
       </c>
       <c r="E10" s="7">
         <v>1</v>
@@ -2631,27 +2631,27 @@
         <v>8</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B11" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="C11" s="7" t="s">
         <v>179</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="D11" s="7" t="s">
         <v>180</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>181</v>
       </c>
       <c r="E11" s="7">
         <v>1</v>
@@ -2660,27 +2660,27 @@
         <v>10</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C12" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>183</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>184</v>
       </c>
       <c r="E12" s="7">
         <v>1</v>
@@ -2689,13 +2689,13 @@
         <v>8</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -2703,7 +2703,7 @@
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
       <c r="D13" s="10" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E13" s="7"/>
       <c r="F13" s="9">

</xml_diff>